<commit_message>
Re-import updated college data spreadsheet and refresh database file
</commit_message>
<xml_diff>
--- a/college_data_template.xlsx
+++ b/college_data_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nanda Kishore\.gemini\antigravity\scratch\student_performance_monitoring\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F2CC5C7-2293-4257-B6EF-8DDA13CF51BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF5DF77-B07D-4C90-8D05-8D4D39B9ACC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="412">
   <si>
     <t xml:space="preserve">  🎓 College Data Import Template — Instructions</t>
   </si>
@@ -1259,9 +1259,6 @@
     <t>23r11a60202</t>
   </si>
   <si>
-    <t>23r11a0202@gcet.edu.in</t>
-  </si>
-  <si>
     <t>aravindailaveni@gmail.com</t>
   </si>
   <si>
@@ -1271,7 +1268,13 @@
     <t>Komuraiah</t>
   </si>
   <si>
-    <t>23r11a0202</t>
+    <t>23r11a60203</t>
+  </si>
+  <si>
+    <t>23r11a0203@gcet.edu.in</t>
+  </si>
+  <si>
+    <t>23r11a0203</t>
   </si>
 </sst>
 </file>
@@ -1463,13 +1466,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1477,33 +1480,10 @@
   </cellStyles>
   <dxfs count="22">
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
       <alignment vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
       <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
       <alignment vertical="center" wrapText="1"/>
@@ -1575,6 +1555,29 @@
       </font>
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1592,9 +1595,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table8" displayName="Table8" ref="A1:C7" totalsRowShown="0">
   <autoFilter ref="A1:C7" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="department_code" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="department_name" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="hod_username" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="department_code" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="department_name" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="hod_username" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1622,19 +1625,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table3" displayName="Table3" ref="A1:M32" totalsRowShown="0">
   <autoFilter ref="A1:M32" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="username" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="password" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="full_name" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="email" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="phone" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="roll_number" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="department_code" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="year" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="section" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="attendance_pct" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="parent_name" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="parent_email" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0200-00000D000000}" name="parent_phone" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="username" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="password" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="full_name" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="email" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="phone" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="roll_number" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="department_code" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="year" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="section" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="attendance_pct" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="parent_name" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="parent_email" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0200-00000D000000}" name="parent_phone" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1644,11 +1647,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table2" displayName="Table2" ref="A1:E146" totalsRowShown="0">
   <autoFilter ref="A1:E146" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="roll_number" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="subject" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="internal_marks" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="assignment_scores" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="exam_marks" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="roll_number" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="subject" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="internal_marks" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="assignment_scores" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="exam_marks" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1659,7 +1662,7 @@
   <autoFilter ref="A1:E100" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="roll_number"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="date" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="date" dataDxfId="21"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="subject"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="status"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Percentage"/>
@@ -1961,10 +1964,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="40.049999999999997" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
+      <c r="B1" s="16"/>
     </row>
     <row r="2" spans="1:2" ht="18" customHeight="1">
       <c r="A2" s="11"/>
@@ -3007,19 +3010,19 @@
         <v>405</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>406</v>
+        <v>407</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>410</v>
       </c>
       <c r="E6" s="7">
         <v>9000000004</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>46</v>
@@ -3034,10 +3037,10 @@
         <v>20</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>409</v>
-      </c>
-      <c r="L6" s="16" t="s">
-        <v>407</v>
+        <v>408</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>406</v>
       </c>
       <c r="M6" s="7">
         <v>9100000004</v>
@@ -4503,7 +4506,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="6" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>370</v>
@@ -4520,7 +4523,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="6" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>371</v>
@@ -4537,7 +4540,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="6" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>373</v>
@@ -4554,7 +4557,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="6" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>372</v>
@@ -7012,7 +7015,7 @@
     </row>
     <row r="15" spans="1:9" ht="16.05" customHeight="1">
       <c r="A15" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B15" s="4">
         <v>46193</v>
@@ -7030,7 +7033,7 @@
     </row>
     <row r="16" spans="1:9" ht="16.05" customHeight="1">
       <c r="A16" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B16" s="4">
         <v>46194</v>
@@ -7048,7 +7051,7 @@
     </row>
     <row r="17" spans="1:9" ht="16.05" customHeight="1">
       <c r="A17" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B17" s="4">
         <v>46195</v>
@@ -7066,7 +7069,7 @@
     </row>
     <row r="18" spans="1:9" ht="16.05" customHeight="1">
       <c r="A18" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B18" s="4">
         <v>46196</v>

</xml_diff>